<commit_message>
feat: automate end-to-end sales analysis pipeline
</commit_message>
<xml_diff>
--- a/data/processed/cleaned_sales_data.xlsx
+++ b/data/processed/cleaned_sales_data.xlsx
@@ -62964,7 +62964,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -63002,67 +63002,67 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Standardize text</t>
+          <t>Handle missing City</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Trimmed text and normalized city/payment spelling</t>
+          <t>Recovered 7 from the same order; labeled 3 as Unknown</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Handle missing City</t>
+          <t>Handle missing Payment_Method</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Recovered 7 from the same order; labeled 3 as Unknown</t>
+          <t>Recovered 4 from the same order; labeled 4 as Unknown</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Handle missing Payment_Method</t>
+          <t>Validate quantity</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Recovered 4 from the same order; labeled 4 as Unknown</t>
+          <t>Removed rows with non-numeric, zero, or negative quantity</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Validate quantity</t>
+          <t>Repair unit prices</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Removed rows with unusable quantity values</t>
+          <t>Replaced with median valid price for the same product</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Repair unit prices</t>
+          <t>Validate discount rates</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -63070,14 +63070,14 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Replaced with median valid price for the same product</t>
+          <t>Removed rows with discount rates outside 0-1</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Validate discount rates</t>
+          <t>Validate order dates</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -63085,14 +63085,14 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Removed rows with discount rates outside 0-1</t>
+          <t>Recovered 4 from the same order; removed 1 unrecoverable rows</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Validate order dates</t>
+          <t>Correct product categories</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -63100,22 +63100,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Recovered 4 from the same order; removed 1 unrecoverable rows</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Correct product categories</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>5</v>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Replaced with approved category for each product</t>
+          <t>Replaced with the approved category for each product</t>
         </is>
       </c>
     </row>

</xml_diff>